<commit_message>
add: T06 from spec 002-s02-architecture
</commit_message>
<xml_diff>
--- a/deliverables/tracking/M4_Equipo06_Proyecto_Integrador_v2.xlsx
+++ b/deliverables/tracking/M4_Equipo06_Proyecto_Integrador_v2.xlsx
@@ -1948,7 +1948,7 @@
           <t>Equipo:</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Grupo 06</t>
         </is>
@@ -1958,7 +1958,7 @@
           <t>Subcaso:</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>03B</t>
         </is>
@@ -1968,7 +1968,7 @@
           <t>Fecha:</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
@@ -3245,7 +3245,7 @@
           <t>Equipo:</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Grupo 06</t>
         </is>
@@ -3255,7 +3255,7 @@
           <t>Subcaso:</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>03B</t>
         </is>
@@ -3265,7 +3265,7 @@
           <t>Fecha:</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
@@ -3626,14 +3626,29 @@
           <t>Equipo:</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Grupo 06</t>
+        </is>
+      </c>
       <c r="C4" s="37" t="inlineStr">
         <is>
           <t>Subcaso:</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>03B</t>
+        </is>
+      </c>
       <c r="E4" s="37" t="inlineStr">
         <is>
           <t>Fecha:</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -3675,77 +3690,189 @@
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="29">
-      <c r="A7" s="52" t="inlineStr">
-        <is>
-          <t>fact_ordenes_silver.csv</t>
-        </is>
-      </c>
-      <c r="B7" s="52" t="inlineStr">
-        <is>
-          <t>Una fila por orden</t>
-        </is>
-      </c>
-      <c r="C7" s="52" t="inlineStr">
-        <is>
-          <t>id_orden (id_activo relaciona)</t>
-        </is>
-      </c>
-      <c r="D7" s="52" t="inlineStr">
-        <is>
-          <t>Diaria</t>
-        </is>
-      </c>
-      <c r="E7" s="52" t="inlineStr">
-        <is>
-          <t>Mantenimiento</t>
-        </is>
-      </c>
-      <c r="F7" s="52" t="inlineStr">
-        <is>
-          <t>Órdenes sin correspondencia de activo</t>
-        </is>
-      </c>
-      <c r="G7" s="52" t="inlineStr">
-        <is>
-          <t>Dimensión gobernada; huérfanas &lt; 1 %</t>
+      <c r="A7" s="43" t="inlineStr">
+        <is>
+          <t>andinalog_iot_telemetry_silver.csv</t>
+        </is>
+      </c>
+      <c r="B7" s="43" t="inlineStr">
+        <is>
+          <t>Una lectura dentro de un viaje</t>
+        </is>
+      </c>
+      <c r="C7" s="43" t="inlineStr">
+        <is>
+          <t>viaje_id + minutos_desde_despacho</t>
+        </is>
+      </c>
+      <c r="D7" s="43" t="inlineStr">
+        <is>
+          <t>Observación cada 30 min; actualización por acordar</t>
+        </is>
+      </c>
+      <c r="E7" s="43" t="inlineStr">
+        <is>
+          <t>Por acordar; revisión Grupo 06</t>
+        </is>
+      </c>
+      <c r="F7" s="43" t="inlineStr">
+        <is>
+          <t>Interpretar el centro del camión como centro real del viaje</t>
+        </is>
+      </c>
+      <c r="G7" s="43" t="inlineStr">
+        <is>
+          <t>Documentar el límite y no usar el centro base como ruta; control de clave compuesta</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="29">
-      <c r="A8" s="43" t="n"/>
-      <c r="B8" s="43" t="n"/>
-      <c r="C8" s="43" t="n"/>
-      <c r="D8" s="43" t="n"/>
-      <c r="E8" s="43" t="n"/>
-      <c r="F8" s="43" t="n"/>
-      <c r="G8" s="43" t="n"/>
+      <c r="A8" s="43" t="inlineStr">
+        <is>
+          <t>andinalog_productos_silver.csv</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="inlineStr">
+        <is>
+          <t>Un producto</t>
+        </is>
+      </c>
+      <c r="C8" s="43" t="inlineStr">
+        <is>
+          <t>producto_id</t>
+        </is>
+      </c>
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>Catálogo; actualización por acordar</t>
+        </is>
+      </c>
+      <c r="E8" s="43" t="inlineStr">
+        <is>
+          <t>Por acordar; revisión Grupo 06</t>
+        </is>
+      </c>
+      <c r="F8" s="43" t="inlineStr">
+        <is>
+          <t>Extrapolar KPI térmicos a todo el catálogo</t>
+        </is>
+      </c>
+      <c r="G8" s="43" t="inlineStr">
+        <is>
+          <t>Registrar cobertura 70 de 120 en telemetría</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="29">
-      <c r="A9" s="43" t="n"/>
-      <c r="B9" s="43" t="n"/>
-      <c r="C9" s="43" t="n"/>
-      <c r="D9" s="43" t="n"/>
-      <c r="E9" s="43" t="n"/>
-      <c r="F9" s="43" t="n"/>
-      <c r="G9" s="43" t="n"/>
+      <c r="A9" s="43" t="inlineStr">
+        <is>
+          <t>andinalog_flota_silver.csv</t>
+        </is>
+      </c>
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>Un camión</t>
+        </is>
+      </c>
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>camion_id</t>
+        </is>
+      </c>
+      <c r="D9" s="43" t="inlineStr">
+        <is>
+          <t>Catálogo; actualización por acordar</t>
+        </is>
+      </c>
+      <c r="E9" s="43" t="inlineStr">
+        <is>
+          <t>Por acordar; revisión Grupo 06</t>
+        </is>
+      </c>
+      <c r="F9" s="43" t="inlineStr">
+        <is>
+          <t>Usar centro_distribucion_base como centro operativo</t>
+        </is>
+      </c>
+      <c r="G9" s="43" t="inlineStr">
+        <is>
+          <t>Mantener la distinción base/operativo y registrarla como pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="29">
-      <c r="A10" s="43" t="n"/>
-      <c r="B10" s="43" t="n"/>
-      <c r="C10" s="43" t="n"/>
-      <c r="D10" s="43" t="n"/>
-      <c r="E10" s="43" t="n"/>
-      <c r="F10" s="43" t="n"/>
-      <c r="G10" s="43" t="n"/>
+      <c r="A10" s="43" t="inlineStr">
+        <is>
+          <t>andinalog_inventory_tracking_silver.csv</t>
+        </is>
+      </c>
+      <c r="B10" s="43" t="inlineStr">
+        <is>
+          <t>Un lote con ingreso, salida y merma en esta entrega</t>
+        </is>
+      </c>
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>lote_id; movimiento_id único en esta entrega</t>
+        </is>
+      </c>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>Sin periodicidad fija: una fila por lote contiene las fechas de ingreso y salida; actualización por acordar</t>
+        </is>
+      </c>
+      <c r="E10" s="43" t="inlineStr">
+        <is>
+          <t>Por acordar; revisión Grupo 06</t>
+        </is>
+      </c>
+      <c r="F10" s="43" t="inlineStr">
+        <is>
+          <t>Leer vencimiento como stock vigente</t>
+        </is>
+      </c>
+      <c r="G10" s="43" t="inlineStr">
+        <is>
+          <t>Declarar que todos los lotes salieron; KPI históricos</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="29">
-      <c r="A11" s="43" t="n"/>
-      <c r="B11" s="43" t="n"/>
-      <c r="C11" s="43" t="n"/>
-      <c r="D11" s="43" t="n"/>
-      <c r="E11" s="43" t="n"/>
-      <c r="F11" s="43" t="n"/>
-      <c r="G11" s="43" t="n"/>
+      <c r="A11" s="43" t="inlineStr">
+        <is>
+          <t>andinalog_warehouse_costs_silver.csv</t>
+        </is>
+      </c>
+      <c r="B11" s="43" t="inlineStr">
+        <is>
+          <t>Un centro en un mes</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>centro_distribucion + periodo_mes</t>
+        </is>
+      </c>
+      <c r="D11" s="43" t="inlineStr">
+        <is>
+          <t>Mensual; actualización por acordar</t>
+        </is>
+      </c>
+      <c r="E11" s="43" t="inlineStr">
+        <is>
+          <t>Por acordar; revisión Grupo 06</t>
+        </is>
+      </c>
+      <c r="F11" s="43" t="inlineStr">
+        <is>
+          <t>Asignar costos a productos sin regla</t>
+        </is>
+      </c>
+      <c r="G11" s="43" t="inlineStr">
+        <is>
+          <t>No asignar; relación temporal en S06</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="29">
       <c r="A12" s="43" t="n"/>

</xml_diff>

<commit_message>
add: T07 from spec 002-s02-architecture
</commit_message>
<xml_diff>
--- a/deliverables/tracking/M4_Equipo06_Proyecto_Integrador_v2.xlsx
+++ b/deliverables/tracking/M4_Equipo06_Proyecto_Integrador_v2.xlsx
@@ -2190,9 +2190,21 @@
           <t>¿Qué proporción de viajes tiene al menos una lectura marcada? Apoya la priorización de controles por producto y camión.</t>
         </is>
       </c>
-      <c r="C7" s="43" t="n"/>
-      <c r="D7" s="43" t="n"/>
-      <c r="E7" s="43" t="n"/>
+      <c r="C7" s="43" t="inlineStr">
+        <is>
+          <t>Táctico</t>
+        </is>
+      </c>
+      <c r="D7" s="43" t="inlineStr">
+        <is>
+          <t>Viajes con al menos una lectura marcada dividido entre viajes observados, multiplicado por 100.</t>
+        </is>
+      </c>
+      <c r="E7" s="43" t="inlineStr">
+        <is>
+          <t>Porcentaje</t>
+        </is>
+      </c>
       <c r="F7" s="43" t="n"/>
       <c r="G7" s="43" t="n"/>
       <c r="H7" s="43" t="n"/>
@@ -2233,9 +2245,21 @@
           <t>¿Qué proporción de lecturas queda marcada? Apoya la lectura de intensidad aparente y la comparación entre productos o camiones.</t>
         </is>
       </c>
-      <c r="C8" s="43" t="n"/>
-      <c r="D8" s="43" t="n"/>
-      <c r="E8" s="43" t="n"/>
+      <c r="C8" s="43" t="inlineStr">
+        <is>
+          <t>Táctico</t>
+        </is>
+      </c>
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>Lecturas marcadas dividido entre lecturas observadas, multiplicado por 100.</t>
+        </is>
+      </c>
+      <c r="E8" s="43" t="inlineStr">
+        <is>
+          <t>Porcentaje</t>
+        </is>
+      </c>
       <c r="F8" s="43" t="n"/>
       <c r="G8" s="43" t="n"/>
       <c r="H8" s="43" t="n"/>
@@ -2276,9 +2300,21 @@
           <t>¿Cuánta cantidad se pierde? Apoya la revisión de lotes y centros con peor desempeño.</t>
         </is>
       </c>
-      <c r="C9" s="43" t="n"/>
-      <c r="D9" s="43" t="n"/>
-      <c r="E9" s="43" t="n"/>
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>Táctico</t>
+        </is>
+      </c>
+      <c r="D9" s="43" t="inlineStr">
+        <is>
+          <t>Suma de cantidad_merma dividida entre suma de cantidad_ingreso, multiplicada por 100.</t>
+        </is>
+      </c>
+      <c r="E9" s="43" t="inlineStr">
+        <is>
+          <t>Porcentaje</t>
+        </is>
+      </c>
       <c r="F9" s="43" t="n"/>
       <c r="G9" s="43" t="n"/>
       <c r="H9" s="43" t="n"/>
@@ -2319,9 +2355,21 @@
           <t>¿Qué proporción de lotes sale vencida? Apoya la revisión de gestión de lotes y centros.</t>
         </is>
       </c>
-      <c r="C10" s="43" t="n"/>
-      <c r="D10" s="43" t="n"/>
-      <c r="E10" s="43" t="n"/>
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>Táctico</t>
+        </is>
+      </c>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>Lotes con salida posterior al día de vencimiento divididos entre lotes salidos, multiplicado por 100.</t>
+        </is>
+      </c>
+      <c r="E10" s="43" t="inlineStr">
+        <is>
+          <t>Porcentaje</t>
+        </is>
+      </c>
       <c r="F10" s="43" t="n"/>
       <c r="G10" s="43" t="n"/>
       <c r="H10" s="43" t="n"/>
@@ -2362,9 +2410,21 @@
           <t>¿Cuánto permanece un lote antes de salir? Apoya la revisión de permanencia histórica por centro o producto.</t>
         </is>
       </c>
-      <c r="C11" s="43" t="n"/>
-      <c r="D11" s="43" t="n"/>
-      <c r="E11" s="43" t="n"/>
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>Táctico</t>
+        </is>
+      </c>
+      <c r="D11" s="43" t="inlineStr">
+        <is>
+          <t>Promedio de dias_en_almacen de los lotes con salida.</t>
+        </is>
+      </c>
+      <c r="E11" s="43" t="inlineStr">
+        <is>
+          <t>Días</t>
+        </is>
+      </c>
       <c r="F11" s="43" t="n"/>
       <c r="G11" s="43" t="n"/>
       <c r="H11" s="43" t="n"/>
@@ -2534,6 +2594,7 @@
         <v/>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="15" customHeight="1" s="29">
       <c r="A17" s="34" t="inlineStr">
         <is>
@@ -3626,7 +3687,7 @@
           <t>Equipo:</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Grupo 06</t>
         </is>
@@ -3636,7 +3697,7 @@
           <t>Subcaso:</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>03B</t>
         </is>
@@ -3646,7 +3707,7 @@
           <t>Fecha:</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>

</xml_diff>

<commit_message>
add: T12 from spec 002-s02-architecture
</commit_message>
<xml_diff>
--- a/deliverables/tracking/M4_Equipo06_Proyecto_Integrador_v2.xlsx
+++ b/deliverables/tracking/M4_Equipo06_Proyecto_Integrador_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\remrodri\Github\Proyecto-Powerbi-Andinalog-rol03b\deliverables\tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B69B4A9-D5E7-44E9-B12D-71170A2F236D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C92C0C20-B52E-468A-8883-7ABBC7AA10C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4160,7 +4160,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>211</v>
       </c>

</xml_diff>